<commit_message>
Re-link updated Almarai & Qassim Cement models to existing portfolio filenames
</commit_message>
<xml_diff>
--- a/models/Almarai-2280-Valuation-Model.xlsx
+++ b/models/Almarai-2280-Valuation-Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Almarai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E42F312-56A0-4DEC-B781-3FA2731DED44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7B7DD1-F88E-48AC-9147-11F0515EAD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="1845" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FSM" sheetId="1" r:id="rId1"/>
@@ -223,7 +223,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="326">
   <si>
     <t>Company Name</t>
   </si>
@@ -1165,6 +1165,42 @@
   </si>
   <si>
     <t>Interest Coverage Ratio EBT / Finance Cost</t>
+  </si>
+  <si>
+    <t>Returns &amp; Profitability</t>
+  </si>
+  <si>
+    <t>Return on Assets (ROA)</t>
+  </si>
+  <si>
+    <t>Return on Equity (ROE)</t>
+  </si>
+  <si>
+    <t>DuPont</t>
+  </si>
+  <si>
+    <t>Net profit margin</t>
+  </si>
+  <si>
+    <t>Asset turnover</t>
+  </si>
+  <si>
+    <t>Equity multiplier (leverage)</t>
+  </si>
+  <si>
+    <t>ROE (DuPont)</t>
+  </si>
+  <si>
+    <t>Check: DuPont = direct ROE</t>
+  </si>
+  <si>
+    <t>Leverage Ratios</t>
+  </si>
+  <si>
+    <t>Coverage Ratios</t>
+  </si>
+  <si>
+    <t>Liquidity Ratios</t>
   </si>
 </sst>
 </file>
@@ -3263,7 +3299,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K340"/>
+  <dimension ref="A1:K356"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="1.7109375" style="6" customWidth="1"/>
@@ -3734,19 +3770,19 @@
       </c>
       <c r="H24" s="235">
         <f t="shared" ref="H24:K24" si="4">H226</f>
-        <v>-462094.22099999996</v>
+        <v>-499561.32</v>
       </c>
       <c r="I24" s="235">
         <f t="shared" si="4"/>
-        <v>-437116.15500000003</v>
+        <v>-499561.32</v>
       </c>
       <c r="J24" s="235">
         <f t="shared" si="4"/>
-        <v>-399649.05599999998</v>
+        <v>-499561.32</v>
       </c>
       <c r="K24" s="235">
         <f t="shared" si="4"/>
-        <v>-374670.99</v>
+        <v>-499561.32</v>
       </c>
     </row>
     <row r="25" spans="3:11" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3800,19 +3836,19 @@
       </c>
       <c r="H26" s="228">
         <f t="shared" si="5"/>
-        <v>2999432.6053977855</v>
+        <v>2961965.5063977856</v>
       </c>
       <c r="I26" s="228">
         <f t="shared" si="5"/>
-        <v>3201611.6830248339</v>
+        <v>3139166.5180248343</v>
       </c>
       <c r="J26" s="228">
         <f t="shared" si="5"/>
-        <v>3400125.6048838878</v>
+        <v>3300213.3408838878</v>
       </c>
       <c r="K26" s="228">
         <f t="shared" si="5"/>
-        <v>3582743.7809260879</v>
+        <v>3457853.4509260883</v>
       </c>
     </row>
     <row r="27" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3837,19 +3873,19 @@
       </c>
       <c r="H27" s="194">
         <f>H26*-H45</f>
-        <v>-160644.55988841734</v>
+        <v>-158637.88515322938</v>
       </c>
       <c r="I27" s="194">
         <f>I26*-I45</f>
-        <v>-171472.93085617776</v>
+        <v>-168128.4729641978</v>
       </c>
       <c r="J27" s="194">
         <f>J26*-J45</f>
-        <v>-182105.00225240839</v>
+        <v>-176753.86962524048</v>
       </c>
       <c r="K27" s="194">
         <f>K26*-K45</f>
-        <v>-191885.72426800913</v>
+        <v>-185196.80848404925</v>
       </c>
     </row>
     <row r="28" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3874,19 +3910,19 @@
       </c>
       <c r="H28" s="228">
         <f t="shared" si="6"/>
-        <v>2838788.0455093682</v>
+        <v>2803327.6212445563</v>
       </c>
       <c r="I28" s="228">
         <f t="shared" si="6"/>
-        <v>3030138.7521686563</v>
+        <v>2971038.0450606365</v>
       </c>
       <c r="J28" s="228">
         <f t="shared" si="6"/>
-        <v>3218020.6026314795</v>
+        <v>3123459.4712586473</v>
       </c>
       <c r="K28" s="228">
         <f t="shared" si="6"/>
-        <v>3390858.0566580789</v>
+        <v>3272656.6424420392</v>
       </c>
     </row>
     <row r="29" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3911,19 +3947,19 @@
       </c>
       <c r="H29" s="235">
         <f t="shared" si="7"/>
-        <v>2838208.0455093682</v>
+        <v>2802747.6212445563</v>
       </c>
       <c r="I29" s="235">
         <f t="shared" si="7"/>
-        <v>3029558.7521686563</v>
+        <v>2970458.0450606365</v>
       </c>
       <c r="J29" s="235">
         <f t="shared" si="7"/>
-        <v>3217440.6026314795</v>
+        <v>3122879.4712586473</v>
       </c>
       <c r="K29" s="235">
         <f t="shared" si="7"/>
-        <v>3390278.0566580789</v>
+        <v>3272076.6424420392</v>
       </c>
     </row>
     <row r="30" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4074,19 +4110,19 @@
       </c>
       <c r="H35" s="243">
         <f>H29/DCF!$I$56</f>
-        <v>2.8688879330655714</v>
+        <v>2.8330441958752464</v>
       </c>
       <c r="I35" s="243">
         <f>I29/DCF!$I$56</f>
-        <v>3.0623070639101111</v>
+        <v>3.0025675019262357</v>
       </c>
       <c r="J35" s="243">
         <f>J29/DCF!$I$56</f>
-        <v>3.2522198416177397</v>
+        <v>3.1566365424435383</v>
       </c>
       <c r="K35" s="243">
         <f>K29/DCF!$I$56</f>
-        <v>3.4269255990139338</v>
+        <v>3.3074464750461829</v>
       </c>
     </row>
     <row r="36" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4108,19 +4144,19 @@
       </c>
       <c r="H36" s="243">
         <f t="shared" si="11"/>
-        <v>2.8382080455093681</v>
+        <v>2.8027476212445563</v>
       </c>
       <c r="I36" s="243">
         <f t="shared" si="11"/>
-        <v>3.0295587521686564</v>
+        <v>2.9704580450606364</v>
       </c>
       <c r="J36" s="243">
         <f t="shared" si="11"/>
-        <v>3.2174406026314797</v>
+        <v>3.1228794712586474</v>
       </c>
       <c r="K36" s="243">
         <f t="shared" si="11"/>
-        <v>3.390278056658079</v>
+        <v>3.2720766424420393</v>
       </c>
     </row>
     <row r="37" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4700,7 +4736,7 @@
       </c>
       <c r="H58" s="19">
         <f t="shared" ref="H58:K58" si="26">H146</f>
-        <v>587381.70289685228</v>
+        <v>587381.70289685205</v>
       </c>
       <c r="I58" s="19">
         <f t="shared" si="26"/>
@@ -4708,11 +4744,11 @@
       </c>
       <c r="J58" s="19">
         <f t="shared" si="26"/>
-        <v>644778.5104288552</v>
+        <v>644778.51042885543</v>
       </c>
       <c r="K58" s="19">
         <f t="shared" si="26"/>
-        <v>671528.24282304058</v>
+        <v>671528.24282304081</v>
       </c>
     </row>
     <row r="59" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5422,19 +5458,19 @@
       </c>
       <c r="H84" s="19">
         <f t="shared" si="44"/>
-        <v>3627292.5545012117</v>
+        <v>3648524.5025334386</v>
       </c>
       <c r="I84" s="19">
         <f t="shared" si="44"/>
-        <v>3978798.9573601219</v>
+        <v>4035417.485446061</v>
       </c>
       <c r="J84" s="19">
         <f t="shared" si="44"/>
-        <v>3451211.1300415932</v>
+        <v>3564448.1862134724</v>
       </c>
       <c r="K84" s="19">
         <f t="shared" si="44"/>
-        <v>2283600.7842758922</v>
+        <v>2467611.0005551949</v>
       </c>
     </row>
     <row r="85" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5459,19 +5495,19 @@
       </c>
       <c r="H85" s="12">
         <f t="shared" si="45"/>
-        <v>10619128.93941194</v>
+        <v>10640360.887444166</v>
       </c>
       <c r="I85" s="12">
         <f t="shared" si="45"/>
-        <v>11254979.094405862</v>
+        <v>11311597.622491799</v>
       </c>
       <c r="J85" s="12">
         <f t="shared" si="45"/>
-        <v>10987452.388145637</v>
+        <v>11100689.444317516</v>
       </c>
       <c r="K85" s="12">
         <f t="shared" si="45"/>
-        <v>10075193.63781983</v>
+        <v>10259203.854099132</v>
       </c>
     </row>
     <row r="86" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5733,19 +5769,19 @@
       </c>
       <c r="H95" s="26">
         <f t="shared" si="52"/>
-        <v>24100504.976388983</v>
+        <v>24121736.924421214</v>
       </c>
       <c r="I95" s="26">
         <f t="shared" si="52"/>
-        <v>24983832.935565241</v>
+        <v>25040451.46365118</v>
       </c>
       <c r="J95" s="26">
         <f t="shared" si="52"/>
-        <v>24986289.493739903</v>
+        <v>25099526.549911782</v>
       </c>
       <c r="K95" s="26">
         <f t="shared" si="52"/>
-        <v>24368557.725855879</v>
+        <v>24552567.942135181</v>
       </c>
     </row>
     <row r="96" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5924,19 +5960,19 @@
       </c>
       <c r="H102" s="19">
         <f t="shared" ref="H102:K102" si="57">H237</f>
-        <v>12369409.265136361</v>
+        <v>12348177.317104133</v>
       </c>
       <c r="I102" s="19">
         <f t="shared" si="57"/>
-        <v>14183359.191574588</v>
+        <v>14126740.663488649</v>
       </c>
       <c r="J102" s="19">
         <f t="shared" si="57"/>
-        <v>16109803.476665592</v>
+        <v>15996566.420493715</v>
       </c>
       <c r="K102" s="19">
         <f t="shared" si="57"/>
-        <v>18139734.279980708</v>
+        <v>17955724.063701406</v>
       </c>
     </row>
     <row r="103" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5961,19 +5997,19 @@
       </c>
       <c r="H103" s="164">
         <f t="shared" ref="H103" si="59">SUM(H98:H102)</f>
-        <v>23792312.265136361</v>
+        <v>23771080.317104131</v>
       </c>
       <c r="I103" s="164">
         <f t="shared" ref="I103" si="60">SUM(I98:I102)</f>
-        <v>25606262.191574588</v>
+        <v>25549643.663488649</v>
       </c>
       <c r="J103" s="164">
         <f t="shared" ref="J103" si="61">SUM(J98:J102)</f>
-        <v>27532706.476665594</v>
+        <v>27419469.420493715</v>
       </c>
       <c r="K103" s="164">
         <f t="shared" ref="K103" si="62">SUM(K98:K102)</f>
-        <v>29562637.279980708</v>
+        <v>29378627.063701406</v>
       </c>
     </row>
     <row r="104" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6032,19 +6068,19 @@
       </c>
       <c r="H105" s="12">
         <f t="shared" ref="H105" si="65">SUM(H103:H104)</f>
-        <v>23793228.265136361</v>
+        <v>23771996.317104131</v>
       </c>
       <c r="I105" s="12">
         <f t="shared" ref="I105" si="66">SUM(I103:I104)</f>
-        <v>25607758.191574588</v>
+        <v>25551139.663488649</v>
       </c>
       <c r="J105" s="12">
         <f t="shared" ref="J105" si="67">SUM(J103:J104)</f>
-        <v>27534782.476665594</v>
+        <v>27421545.420493715</v>
       </c>
       <c r="K105" s="12">
         <f t="shared" ref="K105" si="68">SUM(K103:K104)</f>
-        <v>29565293.279980708</v>
+        <v>29381283.063701406</v>
       </c>
     </row>
     <row r="106" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6223,19 +6259,19 @@
       </c>
       <c r="H115" s="206">
         <f>H28</f>
-        <v>2838788.0455093682</v>
+        <v>2803327.6212445563</v>
       </c>
       <c r="I115" s="206">
         <f>I28</f>
-        <v>3030138.7521686563</v>
+        <v>2971038.0450606365</v>
       </c>
       <c r="J115" s="206">
         <f>J28</f>
-        <v>3218020.6026314795</v>
+        <v>3123459.4712586473</v>
       </c>
       <c r="K115" s="206">
         <f>K28</f>
-        <v>3390858.0566580789</v>
+        <v>3272656.6424420392</v>
       </c>
     </row>
     <row r="116" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6363,19 +6399,19 @@
       </c>
       <c r="H120" s="206">
         <f t="shared" ref="H120:K120" si="77">SUM(H115:H119)</f>
-        <v>5795100.7479797322</v>
+        <v>5759640.3237149203</v>
       </c>
       <c r="I120" s="206">
         <f t="shared" si="77"/>
-        <v>6147023.0145327961</v>
+        <v>6087922.3074247763</v>
       </c>
       <c r="J120" s="206">
         <f t="shared" si="77"/>
-        <v>6484407.6754628196</v>
+        <v>6389846.5440899869</v>
       </c>
       <c r="K120" s="206">
         <f t="shared" si="77"/>
-        <v>6806099.7522847103</v>
+        <v>6687898.3380686706</v>
       </c>
     </row>
     <row r="121" spans="3:11" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6442,19 +6478,19 @@
       </c>
       <c r="H124" s="210">
         <f t="shared" ref="H124:K124" si="79">H120+H123</f>
-        <v>5539649.0679706149</v>
+        <v>5504188.643705803</v>
       </c>
       <c r="I124" s="210">
         <f t="shared" si="79"/>
-        <v>5919399.0750028798</v>
+        <v>5860298.36789486</v>
       </c>
       <c r="J124" s="210">
         <f t="shared" si="79"/>
-        <v>6277534.633760849</v>
+        <v>6182973.5023880163</v>
       </c>
       <c r="K124" s="210">
         <f t="shared" si="79"/>
-        <v>6603602.8108380288</v>
+        <v>6485401.3966219891</v>
       </c>
     </row>
     <row r="125" spans="3:11" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6470,19 +6506,19 @@
       </c>
       <c r="H125" s="206">
         <f t="shared" ref="H125:K125" si="80">SUM(H124)</f>
-        <v>5539649.0679706149</v>
+        <v>5504188.643705803</v>
       </c>
       <c r="I125" s="206">
         <f t="shared" si="80"/>
-        <v>5919399.0750028798</v>
+        <v>5860298.36789486</v>
       </c>
       <c r="J125" s="206">
         <f t="shared" si="80"/>
-        <v>6277534.633760849</v>
+        <v>6182973.5023880163</v>
       </c>
       <c r="K125" s="206">
         <f t="shared" si="80"/>
-        <v>6603602.8108380288</v>
+        <v>6485401.3966219891</v>
       </c>
     </row>
     <row r="126" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6760,19 +6796,19 @@
       </c>
       <c r="H139" s="207">
         <f t="shared" ref="H139:K139" si="88">-H235</f>
-        <v>-1138829.4572305509</v>
+        <v>-1124600.9809979661</v>
       </c>
       <c r="I139" s="207">
         <f t="shared" si="88"/>
-        <v>-1215608.8257304279</v>
+        <v>-1191894.69867612</v>
       </c>
       <c r="J139" s="207">
         <f t="shared" si="88"/>
-        <v>-1290996.3175404754</v>
+        <v>-1253053.7142535825</v>
       </c>
       <c r="K139" s="207">
         <f t="shared" si="88"/>
-        <v>-1360347.2533429624</v>
+        <v>-1312918.9992343467</v>
       </c>
     </row>
     <row r="140" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6816,19 +6852,19 @@
       </c>
       <c r="H141" s="207">
         <f t="shared" ref="H141:K141" si="90">H323</f>
-        <v>1851627.2344203638</v>
+        <v>1872859.1824525907</v>
       </c>
       <c r="I141" s="207">
         <f t="shared" si="90"/>
-        <v>351506.40285891015</v>
+        <v>386892.98291262239</v>
       </c>
       <c r="J141" s="207">
         <f t="shared" si="90"/>
-        <v>-527587.82731852867</v>
+        <v>-470969.29923258862</v>
       </c>
       <c r="K141" s="207">
         <f t="shared" si="90"/>
-        <v>-1167610.345765701</v>
+        <v>-1096837.1856582775</v>
       </c>
     </row>
     <row r="142" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6844,19 +6880,19 @@
       </c>
       <c r="H142" s="210">
         <f t="shared" ref="H142:K142" si="91">SUM(H138:H141)</f>
-        <v>571919.78319395683</v>
+        <v>607380.20745876851</v>
       </c>
       <c r="I142" s="210">
         <f t="shared" si="91"/>
-        <v>-1012192.1833230546</v>
+        <v>-953091.47621503449</v>
       </c>
       <c r="J142" s="210">
         <f t="shared" si="91"/>
-        <v>-1973228.2249739824</v>
+        <v>-1878667.0936011495</v>
       </c>
       <c r="K142" s="210">
         <f t="shared" si="91"/>
-        <v>-2689017.3517259238</v>
+        <v>-2570815.9375098841</v>
       </c>
     </row>
     <row r="143" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6883,15 +6919,15 @@
       </c>
       <c r="H144" s="210">
         <f t="shared" ref="H144:K144" si="92">H125+H134+H142</f>
-        <v>33745.023658484919</v>
+        <v>33745.023658484686</v>
       </c>
       <c r="I144" s="210">
         <f t="shared" si="92"/>
-        <v>30068.994748440571</v>
+        <v>30068.994748440804</v>
       </c>
       <c r="J144" s="210">
         <f t="shared" si="92"/>
-        <v>27327.812783562345</v>
+        <v>27327.812783562578</v>
       </c>
       <c r="K144" s="210">
         <f t="shared" si="92"/>
@@ -6915,7 +6951,7 @@
       </c>
       <c r="I145" s="210">
         <f>H58</f>
-        <v>587381.70289685228</v>
+        <v>587381.70289685205</v>
       </c>
       <c r="J145" s="210">
         <f>I58</f>
@@ -6923,7 +6959,7 @@
       </c>
       <c r="K145" s="210">
         <f>J58</f>
-        <v>644778.5104288552</v>
+        <v>644778.51042885543</v>
       </c>
     </row>
     <row r="146" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6939,7 +6975,7 @@
       </c>
       <c r="H146" s="210">
         <f t="shared" ref="H146:K146" si="93">H144+H145</f>
-        <v>587381.70289685228</v>
+        <v>587381.70289685205</v>
       </c>
       <c r="I146" s="210">
         <f t="shared" si="93"/>
@@ -6947,11 +6983,11 @@
       </c>
       <c r="J146" s="210">
         <f t="shared" si="93"/>
-        <v>644778.5104288552</v>
+        <v>644778.51042885543</v>
       </c>
       <c r="K146" s="210">
         <f t="shared" si="93"/>
-        <v>671528.24282304058</v>
+        <v>671528.24282304081</v>
       </c>
     </row>
     <row r="147" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8791,16 +8827,20 @@
         <v>-0.04</v>
       </c>
       <c r="H219" s="222">
-        <v>-3.6999999999999998E-2</v>
+        <f>G219</f>
+        <v>-0.04</v>
       </c>
       <c r="I219" s="222">
-        <v>-3.5000000000000003E-2</v>
+        <f t="shared" ref="I219:K219" si="140">H219</f>
+        <v>-0.04</v>
       </c>
       <c r="J219" s="222">
-        <v>-3.2000000000000001E-2</v>
+        <f t="shared" si="140"/>
+        <v>-0.04</v>
       </c>
       <c r="K219" s="222">
-        <v>-0.03</v>
+        <f t="shared" si="140"/>
+        <v>-0.04</v>
       </c>
     </row>
     <row r="221" spans="3:11" x14ac:dyDescent="0.25">
@@ -8808,15 +8848,15 @@
         <v>261</v>
       </c>
       <c r="D221" s="191">
-        <f t="shared" ref="D221:F222" si="140">D77</f>
+        <f t="shared" ref="D221:F222" si="141">D77</f>
         <v>844</v>
       </c>
       <c r="E221" s="191">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>52598</v>
       </c>
       <c r="F221" s="191">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>16893</v>
       </c>
       <c r="G221" s="191">
@@ -8824,19 +8864,19 @@
         <v>16893</v>
       </c>
       <c r="H221" s="191">
-        <f t="shared" ref="H221:K221" si="141">G221</f>
+        <f t="shared" ref="H221:K221" si="142">G221</f>
         <v>16893</v>
       </c>
       <c r="I221" s="191">
-        <f t="shared" si="141"/>
+        <f t="shared" si="142"/>
         <v>16893</v>
       </c>
       <c r="J221" s="191">
-        <f t="shared" si="141"/>
+        <f t="shared" si="142"/>
         <v>16893</v>
       </c>
       <c r="K221" s="191">
-        <f t="shared" si="141"/>
+        <f t="shared" si="142"/>
         <v>16893</v>
       </c>
     </row>
@@ -8845,15 +8885,15 @@
         <v>283</v>
       </c>
       <c r="D222" s="191">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>3528828</v>
       </c>
       <c r="E222" s="191">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>1229996</v>
       </c>
       <c r="F222" s="191">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>1520330</v>
       </c>
       <c r="G222" s="191"/>
@@ -8897,7 +8937,7 @@
         <v>0.10662656526925578</v>
       </c>
       <c r="F224" s="217">
-        <f t="shared" ref="F224" si="142">(F221+F222)/F215</f>
+        <f t="shared" ref="F224" si="143">(F221+F222)/F215</f>
         <v>0.15096212362780165</v>
       </c>
       <c r="G224" s="219">
@@ -8905,19 +8945,19 @@
         <v>0.15096212362780165</v>
       </c>
       <c r="H224" s="219">
-        <f t="shared" ref="H224:K224" si="143">G224</f>
+        <f t="shared" ref="H224:K224" si="144">G224</f>
         <v>0.15096212362780165</v>
       </c>
       <c r="I224" s="219">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>0.15096212362780165</v>
       </c>
       <c r="J224" s="219">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>0.15096212362780165</v>
       </c>
       <c r="K224" s="219">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>0.15096212362780165</v>
       </c>
     </row>
@@ -8954,19 +8994,19 @@
       </c>
       <c r="H226" s="191">
         <f>H219*H215</f>
-        <v>-462094.22099999996</v>
+        <v>-499561.32</v>
       </c>
       <c r="I226" s="191">
         <f>I219*I215</f>
-        <v>-437116.15500000003</v>
+        <v>-499561.32</v>
       </c>
       <c r="J226" s="191">
         <f>J219*J215</f>
-        <v>-399649.05599999998</v>
+        <v>-499561.32</v>
       </c>
       <c r="K226" s="191">
         <f>K219*K215</f>
-        <v>-374670.99</v>
+        <v>-499561.32</v>
       </c>
     </row>
     <row r="228" spans="3:11" x14ac:dyDescent="0.25">
@@ -8979,35 +9019,35 @@
         <v>42</v>
       </c>
       <c r="D229" s="52">
-        <f t="shared" ref="D229:K229" si="144">D$13</f>
+        <f t="shared" ref="D229:K229" si="145">D$13</f>
         <v>2023</v>
       </c>
       <c r="E229" s="52">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2024</v>
       </c>
       <c r="F229" s="52">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2025</v>
       </c>
       <c r="G229" s="53">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2026</v>
       </c>
       <c r="H229" s="53">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2027</v>
       </c>
       <c r="I229" s="53">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2028</v>
       </c>
       <c r="J229" s="53">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2029</v>
       </c>
       <c r="K229" s="53">
-        <f t="shared" si="144"/>
+        <f t="shared" si="145"/>
         <v>2030</v>
       </c>
     </row>
@@ -9016,35 +9056,35 @@
         <v>43</v>
       </c>
       <c r="D230" s="245">
-        <f t="shared" ref="D230:K230" si="145">D$14</f>
+        <f t="shared" ref="D230:K230" si="146">D$14</f>
         <v>45291</v>
       </c>
       <c r="E230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>45657</v>
       </c>
       <c r="F230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>46022</v>
       </c>
       <c r="G230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>46387</v>
       </c>
       <c r="H230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>46752</v>
       </c>
       <c r="I230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>47118</v>
       </c>
       <c r="J230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>47483</v>
       </c>
       <c r="K230" s="245">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>47848</v>
       </c>
     </row>
@@ -9063,28 +9103,28 @@
         <v>6403231</v>
       </c>
       <c r="F233" s="191">
-        <f t="shared" ref="F233:K233" si="146">E237</f>
+        <f t="shared" ref="F233:K233" si="147">E237</f>
         <v>7673972</v>
       </c>
       <c r="G233" s="191">
-        <f t="shared" si="146"/>
+        <f t="shared" si="147"/>
         <v>9104577</v>
       </c>
       <c r="H233" s="191">
-        <f t="shared" si="146"/>
+        <f t="shared" si="147"/>
         <v>10670030.676857544</v>
       </c>
       <c r="I233" s="191">
-        <f t="shared" si="146"/>
-        <v>12369409.265136361</v>
+        <f t="shared" si="147"/>
+        <v>12348177.317104133</v>
       </c>
       <c r="J233" s="191">
-        <f t="shared" si="146"/>
-        <v>14183359.191574588</v>
+        <f t="shared" si="147"/>
+        <v>14126740.663488649</v>
       </c>
       <c r="K233" s="191">
-        <f t="shared" si="146"/>
-        <v>16109803.476665592</v>
+        <f t="shared" si="147"/>
+        <v>15996566.420493715</v>
       </c>
     </row>
     <row r="234" spans="3:11" x14ac:dyDescent="0.25">
@@ -9092,36 +9132,36 @@
         <v>170</v>
       </c>
       <c r="D234" s="191">
-        <f t="shared" ref="D234:K234" si="147">D29</f>
+        <f t="shared" ref="D234:K234" si="148">D29</f>
         <v>2049123</v>
       </c>
       <c r="E234" s="191">
-        <f t="shared" si="147"/>
+        <f t="shared" si="148"/>
         <v>2313100</v>
       </c>
       <c r="F234" s="191">
-        <f t="shared" si="147"/>
+        <f t="shared" si="148"/>
         <v>2456093</v>
       </c>
       <c r="G234" s="191">
-        <f t="shared" si="147"/>
+        <f t="shared" si="148"/>
         <v>2614534.0721453903</v>
       </c>
       <c r="H234" s="191">
-        <f t="shared" si="147"/>
-        <v>2838208.0455093682</v>
+        <f t="shared" si="148"/>
+        <v>2802747.6212445563</v>
       </c>
       <c r="I234" s="191">
-        <f t="shared" si="147"/>
-        <v>3029558.7521686563</v>
+        <f t="shared" si="148"/>
+        <v>2970458.0450606365</v>
       </c>
       <c r="J234" s="191">
-        <f t="shared" si="147"/>
-        <v>3217440.6026314795</v>
+        <f t="shared" si="148"/>
+        <v>3122879.4712586473</v>
       </c>
       <c r="K234" s="191">
-        <f t="shared" si="147"/>
-        <v>3390278.0566580789</v>
+        <f t="shared" si="148"/>
+        <v>3272076.6424420392</v>
       </c>
     </row>
     <row r="235" spans="3:11" x14ac:dyDescent="0.25">
@@ -9142,20 +9182,20 @@
         <v>1049080.3952878474</v>
       </c>
       <c r="H235" s="191">
-        <f t="shared" ref="H235:K235" si="148">H234*H245</f>
-        <v>1138829.4572305509</v>
+        <f t="shared" ref="H235:K235" si="149">H234*H245</f>
+        <v>1124600.9809979661</v>
       </c>
       <c r="I235" s="191">
-        <f t="shared" si="148"/>
-        <v>1215608.8257304279</v>
+        <f t="shared" si="149"/>
+        <v>1191894.69867612</v>
       </c>
       <c r="J235" s="191">
-        <f t="shared" si="148"/>
-        <v>1290996.3175404754</v>
+        <f t="shared" si="149"/>
+        <v>1253053.7142535825</v>
       </c>
       <c r="K235" s="191">
-        <f t="shared" si="148"/>
-        <v>1360347.2533429624</v>
+        <f t="shared" si="149"/>
+        <v>1312918.9992343467</v>
       </c>
     </row>
     <row r="236" spans="3:11" x14ac:dyDescent="0.25">
@@ -9192,20 +9232,20 @@
         <v>10670030.676857544</v>
       </c>
       <c r="H237" s="191">
-        <f t="shared" ref="H237:K237" si="149">H233+H234-H235</f>
-        <v>12369409.265136361</v>
+        <f t="shared" ref="H237:K237" si="150">H233+H234-H235</f>
+        <v>12348177.317104133</v>
       </c>
       <c r="I237" s="191">
-        <f t="shared" si="149"/>
-        <v>14183359.191574588</v>
+        <f t="shared" si="150"/>
+        <v>14126740.663488649</v>
       </c>
       <c r="J237" s="191">
-        <f t="shared" si="149"/>
-        <v>16109803.476665592</v>
+        <f t="shared" si="150"/>
+        <v>15996566.420493715</v>
       </c>
       <c r="K237" s="191">
-        <f t="shared" si="149"/>
-        <v>18139734.279980708</v>
+        <f t="shared" si="150"/>
+        <v>17955724.063701406</v>
       </c>
     </row>
     <row r="238" spans="3:11" x14ac:dyDescent="0.25">
@@ -9241,27 +9281,27 @@
         <v>11106</v>
       </c>
       <c r="F240" s="191">
-        <f t="shared" ref="F240:K240" si="150">E243</f>
+        <f t="shared" ref="F240:K240" si="151">E243</f>
         <v>396</v>
       </c>
       <c r="G240" s="191">
-        <f t="shared" si="150"/>
+        <f t="shared" si="151"/>
         <v>-244</v>
       </c>
       <c r="H240" s="191">
-        <f t="shared" si="150"/>
+        <f t="shared" si="151"/>
         <v>336</v>
       </c>
       <c r="I240" s="191">
-        <f t="shared" si="150"/>
+        <f t="shared" si="151"/>
         <v>916</v>
       </c>
       <c r="J240" s="191">
-        <f t="shared" si="150"/>
+        <f t="shared" si="151"/>
         <v>1496</v>
       </c>
       <c r="K240" s="191">
-        <f t="shared" si="150"/>
+        <f t="shared" si="151"/>
         <v>2076</v>
       </c>
     </row>
@@ -9270,35 +9310,35 @@
         <v>175</v>
       </c>
       <c r="D241" s="191">
-        <f t="shared" ref="D241:K241" si="151">D30</f>
+        <f t="shared" ref="D241:K241" si="152">D30</f>
         <v>2406</v>
       </c>
       <c r="E241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>567</v>
       </c>
       <c r="F241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
       <c r="G241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
       <c r="H241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
       <c r="I241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
       <c r="J241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
       <c r="K241" s="191">
-        <f t="shared" si="151"/>
+        <f t="shared" si="152"/>
         <v>580</v>
       </c>
     </row>
@@ -9352,19 +9392,19 @@
         <v>336</v>
       </c>
       <c r="H243" s="191">
-        <f t="shared" ref="H243:K243" si="152">SUM(H240:H242)</f>
+        <f t="shared" ref="H243:K243" si="153">SUM(H240:H242)</f>
         <v>916</v>
       </c>
       <c r="I243" s="191">
-        <f t="shared" si="152"/>
+        <f t="shared" si="153"/>
         <v>1496</v>
       </c>
       <c r="J243" s="191">
-        <f t="shared" si="152"/>
+        <f t="shared" si="153"/>
         <v>2076</v>
       </c>
       <c r="K243" s="191">
-        <f t="shared" si="152"/>
+        <f t="shared" si="153"/>
         <v>2656</v>
       </c>
     </row>
@@ -9387,11 +9427,11 @@
         <v>0.47853447548048605</v>
       </c>
       <c r="E245" s="1">
-        <f t="shared" ref="E245:F245" si="153">E235/E234</f>
+        <f t="shared" ref="E245:F245" si="154">E235/E234</f>
         <v>0.42664605940080413</v>
       </c>
       <c r="F245" s="1">
-        <f t="shared" si="153"/>
+        <f t="shared" si="154"/>
         <v>0.40124946408788265</v>
       </c>
       <c r="G245" s="222">
@@ -9399,19 +9439,19 @@
         <v>0.40124946408788265</v>
       </c>
       <c r="H245" s="222">
-        <f t="shared" ref="H245:K245" si="154">G245</f>
+        <f t="shared" ref="H245:K245" si="155">G245</f>
         <v>0.40124946408788265</v>
       </c>
       <c r="I245" s="222">
-        <f t="shared" si="154"/>
+        <f t="shared" si="155"/>
         <v>0.40124946408788265</v>
       </c>
       <c r="J245" s="222">
-        <f t="shared" si="154"/>
+        <f t="shared" si="155"/>
         <v>0.40124946408788265</v>
       </c>
       <c r="K245" s="222">
-        <f t="shared" si="154"/>
+        <f t="shared" si="155"/>
         <v>0.40124946408788265</v>
       </c>
     </row>
@@ -9436,19 +9476,19 @@
         <v>-9.9344772368147293E-5</v>
       </c>
       <c r="H246" s="222">
-        <f t="shared" ref="H246:K246" si="155">G246</f>
+        <f t="shared" ref="H246:K246" si="156">G246</f>
         <v>-9.9344772368147293E-5</v>
       </c>
       <c r="I246" s="222">
-        <f t="shared" si="155"/>
+        <f t="shared" si="156"/>
         <v>-9.9344772368147293E-5</v>
       </c>
       <c r="J246" s="222">
-        <f t="shared" si="155"/>
+        <f t="shared" si="156"/>
         <v>-9.9344772368147293E-5</v>
       </c>
       <c r="K246" s="222">
-        <f t="shared" si="155"/>
+        <f t="shared" si="156"/>
         <v>-9.9344772368147293E-5</v>
       </c>
     </row>
@@ -9462,35 +9502,35 @@
         <v>42</v>
       </c>
       <c r="D249" s="52">
-        <f t="shared" ref="D249:K249" si="156">D$13</f>
+        <f t="shared" ref="D249:K249" si="157">D$13</f>
         <v>2023</v>
       </c>
       <c r="E249" s="52">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2024</v>
       </c>
       <c r="F249" s="52">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2025</v>
       </c>
       <c r="G249" s="53">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2026</v>
       </c>
       <c r="H249" s="53">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2027</v>
       </c>
       <c r="I249" s="53">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2028</v>
       </c>
       <c r="J249" s="53">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2029</v>
       </c>
       <c r="K249" s="53">
-        <f t="shared" si="156"/>
+        <f t="shared" si="157"/>
         <v>2030</v>
       </c>
     </row>
@@ -9499,35 +9539,35 @@
         <v>43</v>
       </c>
       <c r="D250" s="245">
-        <f t="shared" ref="D250:K250" si="157">D$14</f>
+        <f t="shared" ref="D250:K250" si="158">D$14</f>
         <v>45291</v>
       </c>
       <c r="E250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>45657</v>
       </c>
       <c r="F250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>46022</v>
       </c>
       <c r="G250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>46387</v>
       </c>
       <c r="H250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>46752</v>
       </c>
       <c r="I250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>47118</v>
       </c>
       <c r="J250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>47483</v>
       </c>
       <c r="K250" s="245">
-        <f t="shared" si="157"/>
+        <f t="shared" si="158"/>
         <v>47848</v>
       </c>
     </row>
@@ -9552,27 +9592,27 @@
         <v>1123769</v>
       </c>
       <c r="F252" s="191">
-        <f t="shared" ref="F252:G252" si="158">E255</f>
+        <f t="shared" ref="F252:G252" si="159">E255</f>
         <v>1130692</v>
       </c>
       <c r="G252" s="191">
-        <f t="shared" si="158"/>
+        <f t="shared" si="159"/>
         <v>1612427</v>
       </c>
       <c r="H252" s="191">
-        <f t="shared" ref="H252:K252" si="159">G255</f>
+        <f t="shared" ref="H252:K252" si="160">G255</f>
         <v>1618503.847377552</v>
       </c>
       <c r="I252" s="191">
-        <f t="shared" si="159"/>
+        <f t="shared" si="160"/>
         <v>1624951.0881307861</v>
       </c>
       <c r="J252" s="191">
-        <f t="shared" si="159"/>
+        <f t="shared" si="160"/>
         <v>1631728.3732953372</v>
       </c>
       <c r="K252" s="191">
-        <f t="shared" si="159"/>
+        <f t="shared" si="160"/>
         <v>1638805.6150084257</v>
       </c>
     </row>
@@ -9665,19 +9705,19 @@
         <v>1618503.847377552</v>
       </c>
       <c r="H255" s="191">
-        <f t="shared" ref="H255:K255" si="160">H252+H253-H254</f>
+        <f t="shared" ref="H255:K255" si="161">H252+H253-H254</f>
         <v>1624951.0881307861</v>
       </c>
       <c r="I255" s="191">
-        <f t="shared" si="160"/>
+        <f t="shared" si="161"/>
         <v>1631728.3732953372</v>
       </c>
       <c r="J255" s="191">
-        <f t="shared" si="160"/>
+        <f t="shared" si="161"/>
         <v>1638805.6150084257</v>
       </c>
       <c r="K255" s="191">
-        <f t="shared" si="160"/>
+        <f t="shared" si="161"/>
         <v>1646176.4681227193</v>
       </c>
     </row>
@@ -9702,19 +9742,19 @@
         <v>1.7982426005929062E-3</v>
       </c>
       <c r="H256" s="266">
-        <f t="shared" ref="H256:K256" si="161">G256</f>
+        <f t="shared" ref="H256:K256" si="162">G256</f>
         <v>1.7982426005929062E-3</v>
       </c>
       <c r="I256" s="266">
-        <f t="shared" si="161"/>
+        <f t="shared" si="162"/>
         <v>1.7982426005929062E-3</v>
       </c>
       <c r="J256" s="266">
-        <f t="shared" si="161"/>
+        <f t="shared" si="162"/>
         <v>1.7982426005929062E-3</v>
       </c>
       <c r="K256" s="266">
-        <f t="shared" si="161"/>
+        <f t="shared" si="162"/>
         <v>1.7982426005929062E-3</v>
       </c>
     </row>
@@ -9739,19 +9779,19 @@
         <v>1.5380553237643393E-3</v>
       </c>
       <c r="H257" s="266">
-        <f t="shared" ref="H257:K257" si="162">G257</f>
+        <f t="shared" ref="H257:K257" si="163">G257</f>
         <v>1.5380553237643393E-3</v>
       </c>
       <c r="I257" s="266">
-        <f t="shared" si="162"/>
+        <f t="shared" si="163"/>
         <v>1.5380553237643393E-3</v>
       </c>
       <c r="J257" s="266">
-        <f t="shared" si="162"/>
+        <f t="shared" si="163"/>
         <v>1.5380553237643393E-3</v>
       </c>
       <c r="K257" s="266">
-        <f t="shared" si="162"/>
+        <f t="shared" si="163"/>
         <v>1.5380553237643393E-3</v>
       </c>
     </row>
@@ -9765,35 +9805,35 @@
         <v>42</v>
       </c>
       <c r="D260" s="52">
-        <f t="shared" ref="D260:K260" si="163">D$13</f>
+        <f t="shared" ref="D260:K260" si="164">D$13</f>
         <v>2023</v>
       </c>
       <c r="E260" s="52">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2024</v>
       </c>
       <c r="F260" s="52">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2025</v>
       </c>
       <c r="G260" s="53">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2026</v>
       </c>
       <c r="H260" s="53">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2027</v>
       </c>
       <c r="I260" s="53">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2028</v>
       </c>
       <c r="J260" s="53">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2029</v>
       </c>
       <c r="K260" s="53">
-        <f t="shared" si="163"/>
+        <f t="shared" si="164"/>
         <v>2030</v>
       </c>
     </row>
@@ -9802,35 +9842,35 @@
         <v>43</v>
       </c>
       <c r="D261" s="245">
-        <f t="shared" ref="D261:K261" si="164">D$14</f>
+        <f t="shared" ref="D261:K261" si="165">D$14</f>
         <v>45291</v>
       </c>
       <c r="E261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>45657</v>
       </c>
       <c r="F261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>46022</v>
       </c>
       <c r="G261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>46387</v>
       </c>
       <c r="H261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>46752</v>
       </c>
       <c r="I261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>47118</v>
       </c>
       <c r="J261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>47483</v>
       </c>
       <c r="K261" s="245">
-        <f t="shared" si="164"/>
+        <f t="shared" si="165"/>
         <v>47848</v>
       </c>
     </row>
@@ -9855,27 +9895,27 @@
         <v>473831</v>
       </c>
       <c r="F263" s="191">
-        <f t="shared" ref="F263:G263" si="165">E266</f>
+        <f t="shared" ref="F263:G263" si="166">E266</f>
         <v>504066</v>
       </c>
       <c r="G263" s="191">
-        <f t="shared" si="165"/>
+        <f t="shared" si="166"/>
         <v>551614</v>
       </c>
       <c r="H263" s="191">
-        <f t="shared" ref="H263:K263" si="166">G266</f>
+        <f t="shared" ref="H263:K263" si="167">G266</f>
         <v>607030.69876404142</v>
       </c>
       <c r="I263" s="191">
-        <f t="shared" si="166"/>
+        <f t="shared" si="167"/>
         <v>665825.13220679003</v>
       </c>
       <c r="J263" s="191">
-        <f t="shared" si="166"/>
+        <f t="shared" si="167"/>
         <v>727629.34532382665</v>
       </c>
       <c r="K263" s="191">
-        <f t="shared" si="166"/>
+        <f t="shared" si="167"/>
         <v>792168.95735083101</v>
       </c>
     </row>
@@ -9968,19 +10008,19 @@
         <v>607030.69876404142</v>
       </c>
       <c r="H266" s="191">
-        <f t="shared" ref="H266:K266" si="167">SUM(H263:H265)</f>
+        <f t="shared" ref="H266:K266" si="168">SUM(H263:H265)</f>
         <v>665825.13220679003</v>
       </c>
       <c r="I266" s="191">
-        <f t="shared" si="167"/>
+        <f t="shared" si="168"/>
         <v>727629.34532382665</v>
       </c>
       <c r="J266" s="191">
-        <f t="shared" si="167"/>
+        <f t="shared" si="168"/>
         <v>792168.95735083101</v>
       </c>
       <c r="K266" s="191">
-        <f t="shared" si="167"/>
+        <f t="shared" si="168"/>
         <v>859386.1048766512</v>
       </c>
     </row>
@@ -9993,27 +10033,27 @@
         <v>450192</v>
       </c>
       <c r="F267" s="191">
-        <f t="shared" ref="F267:K267" si="168">E268</f>
+        <f t="shared" ref="F267:K267" si="169">E268</f>
         <v>484950</v>
       </c>
       <c r="G267" s="191">
-        <f t="shared" si="168"/>
+        <f t="shared" si="169"/>
         <v>550226</v>
       </c>
       <c r="H267" s="191">
-        <f t="shared" si="168"/>
+        <f t="shared" si="169"/>
         <v>605642.69876404142</v>
       </c>
       <c r="I267" s="191">
-        <f t="shared" si="168"/>
+        <f t="shared" si="169"/>
         <v>664437.13220679003</v>
       </c>
       <c r="J267" s="191">
-        <f t="shared" si="168"/>
+        <f t="shared" si="169"/>
         <v>726241.34532382665</v>
       </c>
       <c r="K267" s="191">
-        <f t="shared" si="168"/>
+        <f t="shared" si="169"/>
         <v>790780.95735083101</v>
       </c>
     </row>
@@ -10038,19 +10078,19 @@
         <v>605642.69876404142</v>
       </c>
       <c r="H268" s="191">
-        <f t="shared" ref="H268:K268" si="169">H267+H264+H265</f>
+        <f t="shared" ref="H268:K268" si="170">H267+H264+H265</f>
         <v>664437.13220679003</v>
       </c>
       <c r="I268" s="191">
-        <f t="shared" si="169"/>
+        <f t="shared" si="170"/>
         <v>726241.34532382665</v>
       </c>
       <c r="J268" s="191">
-        <f t="shared" si="169"/>
+        <f t="shared" si="170"/>
         <v>790780.95735083101</v>
       </c>
       <c r="K268" s="191">
-        <f t="shared" si="169"/>
+        <f t="shared" si="170"/>
         <v>857998.1048766512</v>
       </c>
     </row>
@@ -10079,15 +10119,15 @@
         <v>0.19582862314757934</v>
       </c>
       <c r="I269" s="217">
-        <f t="shared" ref="I269:K269" si="170">H269</f>
+        <f t="shared" ref="I269:K269" si="171">H269</f>
         <v>0.19582862314757934</v>
       </c>
       <c r="J269" s="217">
-        <f t="shared" si="170"/>
+        <f t="shared" si="171"/>
         <v>0.19582862314757934</v>
       </c>
       <c r="K269" s="217">
-        <f t="shared" si="170"/>
+        <f t="shared" si="171"/>
         <v>0.19582862314757934</v>
       </c>
     </row>
@@ -10112,19 +10152,19 @@
         <v>8.0580557080855569E-3</v>
       </c>
       <c r="H270" s="222">
-        <f t="shared" ref="H270:K270" si="171">G270</f>
+        <f t="shared" ref="H270:K270" si="172">G270</f>
         <v>8.0580557080855569E-3</v>
       </c>
       <c r="I270" s="222">
-        <f t="shared" si="171"/>
+        <f t="shared" si="172"/>
         <v>8.0580557080855569E-3</v>
       </c>
       <c r="J270" s="222">
-        <f t="shared" si="171"/>
+        <f t="shared" si="172"/>
         <v>8.0580557080855569E-3</v>
       </c>
       <c r="K270" s="222">
-        <f t="shared" si="171"/>
+        <f t="shared" si="172"/>
         <v>8.0580557080855569E-3</v>
       </c>
     </row>
@@ -10149,19 +10189,19 @@
         <v>-5.6853254013301503E-3</v>
       </c>
       <c r="H271" s="222">
-        <f t="shared" ref="H271:K271" si="172">G271</f>
+        <f t="shared" ref="H271:K271" si="173">G271</f>
         <v>-5.6853254013301503E-3</v>
       </c>
       <c r="I271" s="222">
-        <f t="shared" si="172"/>
+        <f t="shared" si="173"/>
         <v>-5.6853254013301503E-3</v>
       </c>
       <c r="J271" s="222">
-        <f t="shared" si="172"/>
+        <f t="shared" si="173"/>
         <v>-5.6853254013301503E-3</v>
       </c>
       <c r="K271" s="222">
-        <f t="shared" si="172"/>
+        <f t="shared" si="173"/>
         <v>-5.6853254013301503E-3</v>
       </c>
     </row>
@@ -10175,35 +10215,35 @@
         <v>42</v>
       </c>
       <c r="D274" s="52">
-        <f t="shared" ref="D274:K274" si="173">D$13</f>
+        <f t="shared" ref="D274:K274" si="174">D$13</f>
         <v>2023</v>
       </c>
       <c r="E274" s="52">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2024</v>
       </c>
       <c r="F274" s="52">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2025</v>
       </c>
       <c r="G274" s="53">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2026</v>
       </c>
       <c r="H274" s="53">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2027</v>
       </c>
       <c r="I274" s="53">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2028</v>
       </c>
       <c r="J274" s="53">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2029</v>
       </c>
       <c r="K274" s="53">
-        <f t="shared" si="173"/>
+        <f t="shared" si="174"/>
         <v>2030</v>
       </c>
     </row>
@@ -10212,35 +10252,35 @@
         <v>43</v>
       </c>
       <c r="D275" s="245">
-        <f t="shared" ref="D275:K275" si="174">D$14</f>
+        <f t="shared" ref="D275:K275" si="175">D$14</f>
         <v>45291</v>
       </c>
       <c r="E275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>45657</v>
       </c>
       <c r="F275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>46022</v>
       </c>
       <c r="G275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>46387</v>
       </c>
       <c r="H275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>46752</v>
       </c>
       <c r="I275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>47118</v>
       </c>
       <c r="J275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>47483</v>
       </c>
       <c r="K275" s="245">
-        <f t="shared" si="174"/>
+        <f t="shared" si="175"/>
         <v>47848</v>
       </c>
     </row>
@@ -10254,27 +10294,27 @@
         <v>525153</v>
       </c>
       <c r="F277" s="191">
-        <f t="shared" ref="F277:G277" si="175">E280</f>
+        <f t="shared" ref="F277:G277" si="176">E280</f>
         <v>525391</v>
       </c>
       <c r="G277" s="191">
-        <f t="shared" si="175"/>
+        <f t="shared" si="176"/>
         <v>492514</v>
       </c>
       <c r="H277" s="191">
-        <f t="shared" ref="H277:K277" si="176">G280</f>
+        <f t="shared" ref="H277:K277" si="177">G280</f>
         <v>457713.70192792546</v>
       </c>
       <c r="I277" s="191">
-        <f t="shared" si="176"/>
+        <f t="shared" si="177"/>
         <v>420792.27112421906</v>
       </c>
       <c r="J277" s="191">
-        <f t="shared" si="176"/>
+        <f t="shared" si="177"/>
         <v>381980.77411064209</v>
       </c>
       <c r="K277" s="191">
-        <f t="shared" si="176"/>
+        <f t="shared" si="177"/>
         <v>341451.51513115969</v>
       </c>
     </row>
@@ -10367,19 +10407,19 @@
         <v>457713.70192792546</v>
       </c>
       <c r="H280" s="191">
-        <f t="shared" ref="H280:K280" si="177">H277+H278-H279</f>
+        <f t="shared" ref="H280:K280" si="178">H277+H278-H279</f>
         <v>420792.27112421906</v>
       </c>
       <c r="I280" s="191">
-        <f t="shared" si="177"/>
+        <f t="shared" si="178"/>
         <v>381980.77411064209</v>
       </c>
       <c r="J280" s="191">
-        <f t="shared" si="177"/>
+        <f t="shared" si="178"/>
         <v>341451.51513115969</v>
       </c>
       <c r="K280" s="191">
-        <f t="shared" si="177"/>
+        <f t="shared" si="178"/>
         <v>299240.83095790853</v>
       </c>
     </row>
@@ -10404,19 +10444,19 @@
         <v>5.3297376336943835E-5</v>
       </c>
       <c r="H281" s="222">
-        <f t="shared" ref="H281:K281" si="178">G281</f>
+        <f t="shared" ref="H281:K281" si="179">G281</f>
         <v>5.3297376336943835E-5</v>
       </c>
       <c r="I281" s="222">
-        <f t="shared" si="178"/>
+        <f t="shared" si="179"/>
         <v>5.3297376336943835E-5</v>
       </c>
       <c r="J281" s="222">
-        <f t="shared" si="178"/>
+        <f t="shared" si="179"/>
         <v>5.3297376336943835E-5</v>
       </c>
       <c r="K281" s="222">
-        <f t="shared" si="178"/>
+        <f t="shared" si="179"/>
         <v>5.3297376336943835E-5</v>
       </c>
     </row>
@@ -10441,19 +10481,19 @@
         <v>1.5433125479608406E-3</v>
       </c>
       <c r="H282" s="222">
-        <f t="shared" ref="H282:K282" si="179">G282</f>
+        <f t="shared" ref="H282:K282" si="180">G282</f>
         <v>1.5433125479608406E-3</v>
       </c>
       <c r="I282" s="222">
-        <f t="shared" si="179"/>
+        <f t="shared" si="180"/>
         <v>1.5433125479608406E-3</v>
       </c>
       <c r="J282" s="222">
-        <f t="shared" si="179"/>
+        <f t="shared" si="180"/>
         <v>1.5433125479608406E-3</v>
       </c>
       <c r="K282" s="222">
-        <f t="shared" si="179"/>
+        <f t="shared" si="180"/>
         <v>1.5433125479608406E-3</v>
       </c>
     </row>
@@ -10467,35 +10507,35 @@
         <v>42</v>
       </c>
       <c r="D285" s="52">
-        <f t="shared" ref="D285:K285" si="180">D$13</f>
+        <f t="shared" ref="D285:K285" si="181">D$13</f>
         <v>2023</v>
       </c>
       <c r="E285" s="52">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2024</v>
       </c>
       <c r="F285" s="52">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2025</v>
       </c>
       <c r="G285" s="53">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2026</v>
       </c>
       <c r="H285" s="53">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2027</v>
       </c>
       <c r="I285" s="53">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2028</v>
       </c>
       <c r="J285" s="53">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2029</v>
       </c>
       <c r="K285" s="53">
-        <f t="shared" si="180"/>
+        <f t="shared" si="181"/>
         <v>2030</v>
       </c>
     </row>
@@ -10504,35 +10544,35 @@
         <v>43</v>
       </c>
       <c r="D286" s="245">
-        <f t="shared" ref="D286:K286" si="181">D$14</f>
+        <f t="shared" ref="D286:K286" si="182">D$14</f>
         <v>45291</v>
       </c>
       <c r="E286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>45657</v>
       </c>
       <c r="F286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>46022</v>
       </c>
       <c r="G286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>46387</v>
       </c>
       <c r="H286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>46752</v>
       </c>
       <c r="I286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>47118</v>
       </c>
       <c r="J286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>47483</v>
       </c>
       <c r="K286" s="245">
-        <f t="shared" si="181"/>
+        <f t="shared" si="182"/>
         <v>47848</v>
       </c>
     </row>
@@ -10546,27 +10586,27 @@
         <v>1876863</v>
       </c>
       <c r="F288" s="191">
-        <f t="shared" ref="F288:K288" si="182">E292</f>
+        <f t="shared" ref="F288:K288" si="183">E292</f>
         <v>1974904</v>
       </c>
       <c r="G288" s="191">
-        <f t="shared" si="182"/>
+        <f t="shared" si="183"/>
         <v>1971423</v>
       </c>
       <c r="H288" s="191">
-        <f t="shared" si="182"/>
+        <f t="shared" si="183"/>
         <v>2146463.9142426965</v>
       </c>
       <c r="I288" s="191">
-        <f t="shared" si="182"/>
+        <f t="shared" si="183"/>
         <v>2332173.8466589153</v>
       </c>
       <c r="J288" s="191">
-        <f t="shared" si="182"/>
+        <f t="shared" si="183"/>
         <v>2527390.563088011</v>
       </c>
       <c r="K288" s="191">
-        <f t="shared" si="182"/>
+        <f t="shared" si="183"/>
         <v>2731247.3958845208</v>
       </c>
     </row>
@@ -10735,15 +10775,15 @@
         <v>4.9173593068559257E-2</v>
       </c>
       <c r="I294" s="222">
-        <f t="shared" ref="I294:K296" si="183">H294</f>
+        <f t="shared" ref="I294:K296" si="184">H294</f>
         <v>4.9173593068559257E-2</v>
       </c>
       <c r="J294" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>4.9173593068559257E-2</v>
       </c>
       <c r="K294" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>4.9173593068559257E-2</v>
       </c>
     </row>
@@ -10769,15 +10809,15 @@
         <v>2.7892456727327524E-2</v>
       </c>
       <c r="I295" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>2.7892456727327524E-2</v>
       </c>
       <c r="J295" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>2.7892456727327524E-2</v>
       </c>
       <c r="K295" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>2.7892456727327524E-2</v>
       </c>
     </row>
@@ -10803,15 +10843,15 @@
         <v>1.3786556342624639E-2</v>
       </c>
       <c r="I296" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>1.3786556342624639E-2</v>
       </c>
       <c r="J296" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>1.3786556342624639E-2</v>
       </c>
       <c r="K296" s="222">
-        <f t="shared" si="183"/>
+        <f t="shared" si="184"/>
         <v>1.3786556342624639E-2</v>
       </c>
     </row>
@@ -10846,19 +10886,19 @@
         <v>165433.00697109679</v>
       </c>
       <c r="H298" s="191">
-        <f t="shared" ref="H298:K298" si="184">H292*H301</f>
+        <f t="shared" ref="H298:K298" si="185">H292*H301</f>
         <v>179746.10692127864</v>
       </c>
       <c r="I298" s="191">
-        <f t="shared" si="184"/>
+        <f t="shared" si="185"/>
         <v>194791.91700715816</v>
       </c>
       <c r="J298" s="191">
-        <f t="shared" si="184"/>
+        <f t="shared" si="185"/>
         <v>210503.64112110829</v>
       </c>
       <c r="K298" s="191">
-        <f t="shared" si="184"/>
+        <f t="shared" si="185"/>
         <v>226867.19281414431</v>
       </c>
     </row>
@@ -10883,19 +10923,19 @@
         <v>1981030.9072715996</v>
       </c>
       <c r="H299" s="191">
-        <f t="shared" ref="H299:K299" si="185">H292*H302</f>
+        <f t="shared" ref="H299:K299" si="186">H292*H302</f>
         <v>2152427.7397376369</v>
       </c>
       <c r="I299" s="191">
-        <f t="shared" si="185"/>
+        <f t="shared" si="186"/>
         <v>2332598.646080853</v>
       </c>
       <c r="J299" s="191">
-        <f t="shared" si="185"/>
+        <f t="shared" si="186"/>
         <v>2520743.7547634128</v>
       </c>
       <c r="K299" s="191">
-        <f t="shared" si="185"/>
+        <f t="shared" si="186"/>
         <v>2716694.3830579491</v>
       </c>
     </row>
@@ -10931,15 +10971,15 @@
         <v>7.7072344833462508E-2</v>
       </c>
       <c r="I301" s="222">
-        <f t="shared" ref="I301:K301" si="186">H301</f>
+        <f t="shared" ref="I301:K301" si="187">H301</f>
         <v>7.7072344833462508E-2</v>
       </c>
       <c r="J301" s="222">
-        <f t="shared" si="186"/>
+        <f t="shared" si="187"/>
         <v>7.7072344833462508E-2</v>
       </c>
       <c r="K301" s="222">
-        <f t="shared" si="186"/>
+        <f t="shared" si="187"/>
         <v>7.7072344833462508E-2</v>
       </c>
     </row>
@@ -10961,19 +11001,19 @@
         <v>0.92292765516653752</v>
       </c>
       <c r="H302" s="222">
-        <f t="shared" ref="H302:K302" si="187">1-H301</f>
+        <f t="shared" ref="H302:K302" si="188">1-H301</f>
         <v>0.92292765516653752</v>
       </c>
       <c r="I302" s="222">
-        <f t="shared" si="187"/>
+        <f t="shared" si="188"/>
         <v>0.92292765516653752</v>
       </c>
       <c r="J302" s="222">
-        <f t="shared" si="187"/>
+        <f t="shared" si="188"/>
         <v>0.92292765516653752</v>
       </c>
       <c r="K302" s="222">
-        <f t="shared" si="187"/>
+        <f t="shared" si="188"/>
         <v>0.92292765516653752</v>
       </c>
     </row>
@@ -10997,35 +11037,35 @@
         <v>42</v>
       </c>
       <c r="D305" s="52">
-        <f t="shared" ref="D305:K305" si="188">D$13</f>
+        <f t="shared" ref="D305:K305" si="189">D$13</f>
         <v>2023</v>
       </c>
       <c r="E305" s="52">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2024</v>
       </c>
       <c r="F305" s="52">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2025</v>
       </c>
       <c r="G305" s="53">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2026</v>
       </c>
       <c r="H305" s="53">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2027</v>
       </c>
       <c r="I305" s="53">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2028</v>
       </c>
       <c r="J305" s="53">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2029</v>
       </c>
       <c r="K305" s="53">
-        <f t="shared" si="188"/>
+        <f t="shared" si="189"/>
         <v>2030</v>
       </c>
     </row>
@@ -11034,35 +11074,35 @@
         <v>43</v>
       </c>
       <c r="D306" s="245">
-        <f t="shared" ref="D306:K306" si="189">D$14</f>
+        <f t="shared" ref="D306:K306" si="190">D$14</f>
         <v>45291</v>
       </c>
       <c r="E306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>45657</v>
       </c>
       <c r="F306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>46022</v>
       </c>
       <c r="G306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>46387</v>
       </c>
       <c r="H306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>46752</v>
       </c>
       <c r="I306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>47118</v>
       </c>
       <c r="J306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>47483</v>
       </c>
       <c r="K306" s="245">
-        <f t="shared" si="189"/>
+        <f t="shared" si="190"/>
         <v>47848</v>
       </c>
     </row>
@@ -11076,27 +11116,27 @@
         <v>1225730</v>
       </c>
       <c r="F308" s="191">
-        <f t="shared" ref="F308:K308" si="190">E311</f>
+        <f t="shared" ref="F308:K308" si="191">E311</f>
         <v>1396542</v>
       </c>
       <c r="G308" s="191">
-        <f t="shared" si="190"/>
+        <f t="shared" si="191"/>
         <v>1584310</v>
       </c>
       <c r="H308" s="191">
-        <f t="shared" si="190"/>
+        <f t="shared" si="191"/>
         <v>1746971.144978096</v>
       </c>
       <c r="I308" s="191">
-        <f t="shared" si="190"/>
+        <f t="shared" si="191"/>
         <v>1926332.713538436</v>
       </c>
       <c r="J308" s="191">
-        <f t="shared" si="190"/>
+        <f t="shared" si="191"/>
         <v>2124109.3385631624</v>
       </c>
       <c r="K308" s="191">
-        <f t="shared" si="190"/>
+        <f t="shared" si="191"/>
         <v>2342191.6943327719</v>
       </c>
     </row>
@@ -11116,19 +11156,19 @@
         <v>252641.34747827135</v>
       </c>
       <c r="H309" s="191">
-        <f t="shared" ref="H309:K309" si="191">H313*H308</f>
+        <f t="shared" ref="H309:K309" si="192">H313*H308</f>
         <v>278580.0405684018</v>
       </c>
       <c r="I309" s="191">
-        <f t="shared" si="191"/>
+        <f t="shared" si="192"/>
         <v>307181.85988842166</v>
       </c>
       <c r="J309" s="191">
-        <f t="shared" si="191"/>
+        <f t="shared" si="192"/>
         <v>338720.22867101576</v>
       </c>
       <c r="K309" s="191">
-        <f t="shared" si="191"/>
+        <f t="shared" si="192"/>
         <v>373496.64251860237</v>
       </c>
     </row>
@@ -11148,19 +11188,19 @@
         <v>89980.202500175423</v>
       </c>
       <c r="H310" s="191">
-        <f t="shared" ref="H310:K310" si="192">H314*H308</f>
+        <f t="shared" ref="H310:K310" si="193">H314*H308</f>
         <v>99218.472008061814</v>
       </c>
       <c r="I310" s="191">
-        <f t="shared" si="192"/>
+        <f t="shared" si="193"/>
         <v>109405.23486369516</v>
       </c>
       <c r="J310" s="191">
-        <f t="shared" si="192"/>
+        <f t="shared" si="193"/>
         <v>120637.87290140631</v>
       </c>
       <c r="K310" s="191">
-        <f t="shared" si="192"/>
+        <f t="shared" si="193"/>
         <v>133023.76615074815</v>
       </c>
     </row>
@@ -11185,19 +11225,19 @@
         <v>1746971.144978096</v>
       </c>
       <c r="H311" s="191">
-        <f t="shared" ref="H311:K311" si="193">H308+H309-H310</f>
+        <f t="shared" ref="H311:K311" si="194">H308+H309-H310</f>
         <v>1926332.713538436</v>
       </c>
       <c r="I311" s="191">
-        <f t="shared" si="193"/>
+        <f t="shared" si="194"/>
         <v>2124109.3385631624</v>
       </c>
       <c r="J311" s="191">
-        <f t="shared" si="193"/>
+        <f t="shared" si="194"/>
         <v>2342191.6943327719</v>
       </c>
       <c r="K311" s="191">
-        <f t="shared" si="193"/>
+        <f t="shared" si="194"/>
         <v>2582664.5707006259</v>
       </c>
     </row>
@@ -11219,19 +11259,19 @@
         <v>0.15946459182752828</v>
       </c>
       <c r="H313" s="219">
-        <f t="shared" ref="H313:K313" si="194">G313</f>
+        <f t="shared" ref="H313:K313" si="195">G313</f>
         <v>0.15946459182752828</v>
       </c>
       <c r="I313" s="219">
-        <f t="shared" si="194"/>
+        <f t="shared" si="195"/>
         <v>0.15946459182752828</v>
       </c>
       <c r="J313" s="219">
-        <f t="shared" si="194"/>
+        <f t="shared" si="195"/>
         <v>0.15946459182752828</v>
       </c>
       <c r="K313" s="219">
-        <f t="shared" si="194"/>
+        <f t="shared" si="195"/>
         <v>0.15946459182752828</v>
       </c>
     </row>
@@ -11253,19 +11293,19 @@
         <v>5.6794568297981726E-2</v>
       </c>
       <c r="H314" s="219">
-        <f t="shared" ref="H314:K314" si="195">G314</f>
+        <f t="shared" ref="H314:K314" si="196">G314</f>
         <v>5.6794568297981726E-2</v>
       </c>
       <c r="I314" s="219">
-        <f t="shared" si="195"/>
+        <f t="shared" si="196"/>
         <v>5.6794568297981726E-2</v>
       </c>
       <c r="J314" s="219">
-        <f t="shared" si="195"/>
+        <f t="shared" si="196"/>
         <v>5.6794568297981726E-2</v>
       </c>
       <c r="K314" s="219">
-        <f t="shared" si="195"/>
+        <f t="shared" si="196"/>
         <v>5.6794568297981726E-2</v>
       </c>
     </row>
@@ -11279,35 +11319,35 @@
         <v>42</v>
       </c>
       <c r="D317" s="52">
-        <f t="shared" ref="D317:K317" si="196">D$13</f>
+        <f t="shared" ref="D317:K317" si="197">D$13</f>
         <v>2023</v>
       </c>
       <c r="E317" s="52">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2024</v>
       </c>
       <c r="F317" s="52">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2025</v>
       </c>
       <c r="G317" s="53">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2026</v>
       </c>
       <c r="H317" s="53">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2027</v>
       </c>
       <c r="I317" s="53">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2028</v>
       </c>
       <c r="J317" s="53">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2029</v>
       </c>
       <c r="K317" s="53">
-        <f t="shared" si="196"/>
+        <f t="shared" si="197"/>
         <v>2030</v>
       </c>
     </row>
@@ -11316,35 +11356,35 @@
         <v>43</v>
       </c>
       <c r="D318" s="245">
-        <f t="shared" ref="D318:K318" si="197">D$14</f>
+        <f t="shared" ref="D318:K318" si="198">D$14</f>
         <v>45291</v>
       </c>
       <c r="E318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>45657</v>
       </c>
       <c r="F318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>46022</v>
       </c>
       <c r="G318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>46387</v>
       </c>
       <c r="H318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>46752</v>
       </c>
       <c r="I318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>47118</v>
       </c>
       <c r="J318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>47483</v>
       </c>
       <c r="K318" s="245">
-        <f t="shared" si="197"/>
+        <f t="shared" si="198"/>
         <v>47848</v>
       </c>
     </row>
@@ -11353,35 +11393,35 @@
         <v>301</v>
       </c>
       <c r="D320" s="191">
-        <f t="shared" ref="D320:K320" si="198">D324*D16</f>
+        <f t="shared" ref="D320:K320" si="199">D324*D16</f>
         <v>666336</v>
       </c>
       <c r="E320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>528214</v>
       </c>
       <c r="F320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>523038.99999999994</v>
       </c>
       <c r="G320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>553636.67923836736</v>
       </c>
       <c r="H320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>587381.70289685216</v>
       </c>
       <c r="I320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>617450.69764529273</v>
       </c>
       <c r="J320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>644778.51042885531</v>
       </c>
       <c r="K320" s="191">
-        <f t="shared" si="198"/>
+        <f t="shared" si="199"/>
         <v>671528.24282304081</v>
       </c>
     </row>
@@ -11397,20 +11437,20 @@
         <v>-1222028.6408424806</v>
       </c>
       <c r="H321" s="191">
-        <f t="shared" ref="H321:K321" si="199">H125+H134+H138+H139+H140+H145</f>
-        <v>-1264245.5315235115</v>
+        <f t="shared" ref="H321:K321" si="200">H125+H134+H138+H139+H140+H145</f>
+        <v>-1285477.4795557386</v>
       </c>
       <c r="I321" s="191">
-        <f t="shared" si="199"/>
-        <v>265944.2947863827</v>
+        <f t="shared" si="200"/>
+        <v>230557.71473267046</v>
       </c>
       <c r="J321" s="191">
-        <f t="shared" si="199"/>
-        <v>1172366.3377473839</v>
+        <f t="shared" si="200"/>
+        <v>1115747.809661444</v>
       </c>
       <c r="K321" s="191">
-        <f t="shared" si="199"/>
-        <v>1839138.5885887418</v>
+        <f t="shared" si="200"/>
+        <v>1768365.4284813181</v>
       </c>
     </row>
     <row r="322" spans="3:11" x14ac:dyDescent="0.25">
@@ -11426,19 +11466,19 @@
       </c>
       <c r="H322" s="191">
         <f>MAX(0, G322 - (H321 - H320))</f>
-        <v>3627292.5545012117</v>
+        <v>3648524.5025334386</v>
       </c>
       <c r="I322" s="191">
         <f>MAX(0, H322 - (I321 - I320))</f>
-        <v>3978798.9573601219</v>
+        <v>4035417.485446061</v>
       </c>
       <c r="J322" s="191">
-        <f t="shared" ref="J322:K322" si="200">MAX(0, I322 - (J321 - J320))</f>
-        <v>3451211.1300415932</v>
+        <f t="shared" ref="J322:K322" si="201">MAX(0, I322 - (J321 - J320))</f>
+        <v>3564448.1862134724</v>
       </c>
       <c r="K322" s="191">
-        <f t="shared" si="200"/>
-        <v>2283600.7842758922</v>
+        <f t="shared" si="201"/>
+        <v>2467611.0005551949</v>
       </c>
     </row>
     <row r="323" spans="3:11" x14ac:dyDescent="0.25">
@@ -11453,20 +11493,20 @@
         <v>1775665.3200808479</v>
       </c>
       <c r="H323" s="191">
-        <f t="shared" ref="H323:K323" si="201">H322 - G322</f>
-        <v>1851627.2344203638</v>
+        <f t="shared" ref="H323:K323" si="202">H322 - G322</f>
+        <v>1872859.1824525907</v>
       </c>
       <c r="I323" s="191">
-        <f t="shared" si="201"/>
-        <v>351506.40285891015</v>
+        <f t="shared" si="202"/>
+        <v>386892.98291262239</v>
       </c>
       <c r="J323" s="191">
-        <f t="shared" si="201"/>
-        <v>-527587.82731852867</v>
+        <f t="shared" si="202"/>
+        <v>-470969.29923258862</v>
       </c>
       <c r="K323" s="191">
-        <f t="shared" si="201"/>
-        <v>-1167610.345765701</v>
+        <f t="shared" si="202"/>
+        <v>-1096837.1856582775</v>
       </c>
     </row>
     <row r="324" spans="3:11" x14ac:dyDescent="0.25">
@@ -11490,19 +11530,19 @@
         <v>2.3704597297532964E-2</v>
       </c>
       <c r="H324" s="222">
-        <f t="shared" ref="H324:K324" si="202">G324</f>
+        <f t="shared" ref="H324:K324" si="203">G324</f>
         <v>2.3704597297532964E-2</v>
       </c>
       <c r="I324" s="222">
-        <f t="shared" si="202"/>
+        <f t="shared" si="203"/>
         <v>2.3704597297532964E-2</v>
       </c>
       <c r="J324" s="222">
-        <f t="shared" si="202"/>
+        <f t="shared" si="203"/>
         <v>2.3704597297532964E-2</v>
       </c>
       <c r="K324" s="222">
-        <f t="shared" si="202"/>
+        <f t="shared" si="203"/>
         <v>2.3704597297532964E-2</v>
       </c>
     </row>
@@ -11517,35 +11557,35 @@
         <v>42</v>
       </c>
       <c r="D327" s="52">
-        <f t="shared" ref="D327:K327" si="203">D$13</f>
+        <f t="shared" ref="D327:K327" si="204">D$13</f>
         <v>2023</v>
       </c>
       <c r="E327" s="52">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2024</v>
       </c>
       <c r="F327" s="52">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2025</v>
       </c>
       <c r="G327" s="53">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2026</v>
       </c>
       <c r="H327" s="53">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2027</v>
       </c>
       <c r="I327" s="53">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2028</v>
       </c>
       <c r="J327" s="53">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2029</v>
       </c>
       <c r="K327" s="53">
-        <f t="shared" si="203"/>
+        <f t="shared" si="204"/>
         <v>2030</v>
       </c>
     </row>
@@ -11554,35 +11594,35 @@
         <v>43</v>
       </c>
       <c r="D328" s="271">
-        <f t="shared" ref="D328:K328" si="204">D$14</f>
+        <f t="shared" ref="D328:K328" si="205">D$14</f>
         <v>45291</v>
       </c>
       <c r="E328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>45657</v>
       </c>
       <c r="F328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>46022</v>
       </c>
       <c r="G328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>46387</v>
       </c>
       <c r="H328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>46752</v>
       </c>
       <c r="I328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>47118</v>
       </c>
       <c r="J328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>47483</v>
       </c>
       <c r="K328" s="245">
-        <f t="shared" si="204"/>
+        <f t="shared" si="205"/>
         <v>47848</v>
       </c>
     </row>
@@ -11598,32 +11638,32 @@
         <v>12478189</v>
       </c>
       <c r="E330" s="165">
-        <f t="shared" ref="E330:K330" si="205">E78+E79+E88+E89+E84</f>
+        <f t="shared" ref="E330:K330" si="206">E78+E79+E88+E89+E84</f>
         <v>10615191</v>
       </c>
       <c r="F330" s="165">
-        <f t="shared" si="205"/>
+        <f t="shared" si="206"/>
         <v>13022366</v>
       </c>
       <c r="G330" s="165">
-        <f t="shared" si="205"/>
+        <f t="shared" si="206"/>
         <v>14853448.018844889</v>
       </c>
       <c r="H330" s="165">
-        <f t="shared" si="205"/>
-        <v>16763869.686708001</v>
+        <f t="shared" si="206"/>
+        <v>16785101.63474023</v>
       </c>
       <c r="I330" s="165">
-        <f t="shared" si="205"/>
-        <v>17177180.302683949</v>
+        <f t="shared" si="206"/>
+        <v>17233798.830769889</v>
       </c>
       <c r="J330" s="165">
-        <f t="shared" si="205"/>
-        <v>16714132.087392425</v>
+        <f t="shared" si="206"/>
+        <v>16827369.143564302</v>
       </c>
       <c r="K330" s="165">
-        <f t="shared" si="205"/>
-        <v>15613738.889152542</v>
+        <f t="shared" si="206"/>
+        <v>15797749.105431845</v>
       </c>
     </row>
     <row r="331" spans="3:11" x14ac:dyDescent="0.25">
@@ -11635,120 +11675,97 @@
         <v>11811853</v>
       </c>
       <c r="E331" s="165">
-        <f t="shared" ref="E331:K331" si="206">E330-E58</f>
+        <f t="shared" ref="E331:K331" si="207">E330-E58</f>
         <v>10086977</v>
       </c>
       <c r="F331" s="165">
-        <f t="shared" si="206"/>
+        <f t="shared" si="207"/>
         <v>12499327</v>
       </c>
       <c r="G331" s="165">
-        <f t="shared" si="206"/>
+        <f t="shared" si="207"/>
         <v>14299811.339606522</v>
       </c>
       <c r="H331" s="165">
-        <f t="shared" si="206"/>
-        <v>16176487.983811149</v>
+        <f t="shared" si="207"/>
+        <v>16197719.931843378</v>
       </c>
       <c r="I331" s="165">
-        <f t="shared" si="206"/>
-        <v>16559729.605038656</v>
+        <f t="shared" si="207"/>
+        <v>16616348.133124596</v>
       </c>
       <c r="J331" s="165">
-        <f t="shared" si="206"/>
-        <v>16069353.57696357</v>
+        <f t="shared" si="207"/>
+        <v>16182590.633135447</v>
       </c>
       <c r="K331" s="165">
-        <f t="shared" si="206"/>
-        <v>14942210.646329502</v>
+        <f t="shared" si="207"/>
+        <v>15126220.862608805</v>
       </c>
     </row>
     <row r="332" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D332" s="30"/>
-      <c r="E332" s="30"/>
-      <c r="F332" s="30"/>
-      <c r="G332" s="30"/>
-      <c r="H332" s="30"/>
-      <c r="I332" s="30"/>
-      <c r="J332" s="30"/>
-      <c r="K332" s="30"/>
+      <c r="C332" s="13"/>
+      <c r="D332" s="165"/>
+      <c r="E332" s="165"/>
+      <c r="F332" s="165"/>
+      <c r="G332" s="165"/>
+      <c r="H332" s="165"/>
+      <c r="I332" s="165"/>
+      <c r="J332" s="165"/>
+      <c r="K332" s="165"/>
     </row>
     <row r="333" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C333" s="6" t="s">
+      <c r="C333" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="D333" s="30"/>
+      <c r="E333" s="30"/>
+      <c r="F333" s="30"/>
+      <c r="G333" s="30"/>
+      <c r="H333" s="30"/>
+      <c r="I333" s="30"/>
+      <c r="J333" s="30"/>
+      <c r="K333" s="30"/>
+    </row>
+    <row r="334" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C334" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="D333" s="272">
+      <c r="D334" s="272">
         <f>D331/D32</f>
         <v>2.2911346417196525</v>
       </c>
-      <c r="E333" s="272">
-        <f t="shared" ref="E333:K333" si="207">E331/E32</f>
+      <c r="E334" s="272">
+        <f t="shared" ref="E334:K334" si="208">E331/E32</f>
         <v>1.8558486042098992</v>
-      </c>
-      <c r="F333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.2463511900910809</v>
-      </c>
-      <c r="G333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.4319084491868606</v>
-      </c>
-      <c r="H333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.5930183751122837</v>
-      </c>
-      <c r="I333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.5251822292963007</v>
-      </c>
-      <c r="J333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.3465489650594966</v>
-      </c>
-      <c r="K333" s="272">
-        <f t="shared" si="207"/>
-        <v>2.0950401034113315</v>
-      </c>
-    </row>
-    <row r="334" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C334" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="D334" s="272">
-        <f>D23/ABS(D24)</f>
-        <v>5.1115576478267384</v>
-      </c>
-      <c r="E334" s="272">
-        <f t="shared" ref="E334:K334" si="208">E23/ABS(E24)</f>
-        <v>5.6488533926752913</v>
       </c>
       <c r="F334" s="272">
         <f t="shared" si="208"/>
-        <v>6.6047014542048492</v>
+        <v>2.2463511900910809</v>
       </c>
       <c r="G334" s="272">
         <f t="shared" si="208"/>
-        <v>6.531054957104133</v>
+        <v>2.4319084491868606</v>
       </c>
       <c r="H334" s="272">
         <f t="shared" si="208"/>
-        <v>7.4909545912667577</v>
+        <v>2.5964217610290596</v>
       </c>
       <c r="I334" s="272">
         <f t="shared" si="208"/>
-        <v>8.3243956930048348</v>
+        <v>2.5338159512459648</v>
       </c>
       <c r="J334" s="272">
         <f t="shared" si="208"/>
-        <v>9.5077783966638165</v>
+        <v>2.3630845584605544</v>
       </c>
       <c r="K334" s="272">
         <f t="shared" si="208"/>
-        <v>10.562373059430323</v>
+        <v>2.1208400865374717</v>
       </c>
     </row>
     <row r="335" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C335" s="6" t="s">
+      <c r="C335" s="17" t="s">
         <v>307</v>
       </c>
       <c r="D335" s="1">
@@ -11769,176 +11786,532 @@
       </c>
       <c r="H335" s="1">
         <f t="shared" si="209"/>
-        <v>0.35002219605994733</v>
+        <v>0.35046550975873875</v>
       </c>
       <c r="I335" s="1">
         <f t="shared" si="209"/>
-        <v>0.3395263900579174</v>
+        <v>0.34064551928126313</v>
       </c>
       <c r="J335" s="1">
         <f t="shared" si="209"/>
-        <v>0.31823668977682873</v>
+        <v>0.32039272071686137</v>
       </c>
       <c r="K335" s="1">
         <f t="shared" si="209"/>
-        <v>0.28949794234909831</v>
+        <v>0.29290971830886409</v>
       </c>
     </row>
     <row r="336" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C336" s="6" t="s">
+      <c r="C336" s="17" t="s">
         <v>308</v>
       </c>
       <c r="D336" s="1">
-        <f>D331/D102</f>
-        <v>1.8446707607456299</v>
+        <f>D331/D105</f>
+        <v>0.66325841261284779</v>
       </c>
       <c r="E336" s="1">
-        <f t="shared" ref="E336:K336" si="210">E331/E102</f>
-        <v>1.3144401621481028</v>
+        <f t="shared" ref="E336:K336" si="210">E331/E105</f>
+        <v>0.53679453691241164</v>
       </c>
       <c r="F336" s="1">
         <f t="shared" si="210"/>
-        <v>1.3728619132992121</v>
+        <v>0.60891427369958628</v>
       </c>
       <c r="G336" s="1">
         <f t="shared" si="210"/>
-        <v>1.3401846510733737</v>
+        <v>0.64724739926500852</v>
       </c>
       <c r="H336" s="1">
         <f t="shared" si="210"/>
-        <v>1.3077817733305326</v>
+        <v>0.6813781945687496</v>
       </c>
       <c r="I336" s="1">
         <f t="shared" si="210"/>
-        <v>1.1675463746892707</v>
+        <v>0.65031729903103141</v>
       </c>
       <c r="J336" s="1">
         <f t="shared" si="210"/>
-        <v>0.99748911277778085</v>
+        <v>0.59014145209486468</v>
       </c>
       <c r="K336" s="1">
         <f t="shared" si="210"/>
-        <v>0.82372819886452009</v>
+        <v>0.51482506158133823</v>
       </c>
     </row>
     <row r="337" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C337" s="6" t="s">
+      <c r="E337" s="7"/>
+      <c r="F337" s="7"/>
+      <c r="G337" s="7"/>
+      <c r="H337" s="7"/>
+      <c r="I337" s="7"/>
+      <c r="J337" s="7"/>
+      <c r="K337" s="7"/>
+    </row>
+    <row r="338" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C338" s="13" t="s">
+        <v>324</v>
+      </c>
+      <c r="E338" s="7"/>
+      <c r="F338" s="7"/>
+      <c r="G338" s="7"/>
+      <c r="H338" s="7"/>
+      <c r="I338" s="7"/>
+      <c r="J338" s="7"/>
+      <c r="K338" s="7"/>
+    </row>
+    <row r="339" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C339" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="D339" s="272">
+        <f>D23/ABS(D24)</f>
+        <v>5.1115576478267384</v>
+      </c>
+      <c r="E339" s="272">
+        <f t="shared" ref="E339:K339" si="211">E23/ABS(E24)</f>
+        <v>5.6488533926752913</v>
+      </c>
+      <c r="F339" s="272">
+        <f t="shared" si="211"/>
+        <v>6.6047014542048492</v>
+      </c>
+      <c r="G339" s="272">
+        <f t="shared" si="211"/>
+        <v>6.531054957104133</v>
+      </c>
+      <c r="H339" s="272">
+        <f t="shared" si="211"/>
+        <v>6.9291329969217497</v>
+      </c>
+      <c r="I339" s="272">
+        <f t="shared" si="211"/>
+        <v>7.2838462313792309</v>
+      </c>
+      <c r="J339" s="272">
+        <f t="shared" si="211"/>
+        <v>7.606222717331053</v>
+      </c>
+      <c r="K339" s="272">
+        <f t="shared" si="211"/>
+        <v>7.9217797945727426</v>
+      </c>
+    </row>
+    <row r="341" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C341" s="204" t="s">
+        <v>325</v>
+      </c>
+      <c r="D341" s="1"/>
+      <c r="E341" s="1"/>
+      <c r="F341" s="1"/>
+      <c r="G341" s="1"/>
+      <c r="H341" s="1"/>
+      <c r="I341" s="1"/>
+      <c r="J341" s="1"/>
+      <c r="K341" s="1"/>
+    </row>
+    <row r="342" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C342" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="D337" s="272">
+      <c r="D342" s="272">
         <f>D59/D85</f>
         <v>1.399231239882204</v>
       </c>
-      <c r="E337" s="272">
-        <f t="shared" ref="E337:K337" si="211">E59/E85</f>
+      <c r="E342" s="272">
+        <f t="shared" ref="E342:K342" si="212">E59/E85</f>
         <v>1.5044895744521238</v>
       </c>
-      <c r="F337" s="272">
-        <f t="shared" si="211"/>
+      <c r="F342" s="272">
+        <f t="shared" si="212"/>
         <v>1.4692399463467245</v>
       </c>
-      <c r="G337" s="272">
-        <f t="shared" si="211"/>
+      <c r="G342" s="272">
+        <f t="shared" si="212"/>
         <v>1.1748980921729055</v>
       </c>
-      <c r="H337" s="272">
-        <f t="shared" si="211"/>
-        <v>0.99231002419272019</v>
-      </c>
-      <c r="I337" s="272">
-        <f t="shared" si="211"/>
-        <v>0.98467064792876258</v>
-      </c>
-      <c r="J337" s="272">
-        <f t="shared" si="211"/>
-        <v>1.0539096912131136</v>
-      </c>
-      <c r="K337" s="272">
-        <f t="shared" si="211"/>
-        <v>1.1977518017949045</v>
-      </c>
-    </row>
-    <row r="338" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C338" s="6" t="s">
+      <c r="H342" s="272">
+        <f t="shared" si="212"/>
+        <v>0.9903299527375895</v>
+      </c>
+      <c r="I342" s="272">
+        <f t="shared" si="212"/>
+        <v>0.9797420247054347</v>
+      </c>
+      <c r="J342" s="272">
+        <f t="shared" si="212"/>
+        <v>1.043158860690143</v>
+      </c>
+      <c r="K342" s="272">
+        <f t="shared" si="212"/>
+        <v>1.1762687928566289</v>
+      </c>
+    </row>
+    <row r="343" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C343" s="17" t="s">
         <v>310</v>
       </c>
-      <c r="D338" s="272">
+      <c r="D343" s="272">
         <f>(D59-D53)/D85</f>
         <v>0.6482330035988908</v>
       </c>
-      <c r="E338" s="272">
-        <f t="shared" ref="E338:K338" si="212">(E59-E53)/E85</f>
+      <c r="E343" s="272">
+        <f t="shared" ref="E343:K343" si="213">(E59-E53)/E85</f>
         <v>0.53090292633316194</v>
       </c>
-      <c r="F338" s="272">
-        <f t="shared" si="212"/>
+      <c r="F343" s="272">
+        <f t="shared" si="213"/>
         <v>0.52969155624223074</v>
       </c>
-      <c r="G338" s="272">
-        <f t="shared" si="212"/>
+      <c r="G343" s="272">
+        <f t="shared" si="213"/>
         <v>0.4235150533642934</v>
       </c>
-      <c r="H338" s="272">
-        <f t="shared" si="212"/>
-        <v>0.35793122097829905</v>
-      </c>
-      <c r="I338" s="272">
-        <f t="shared" si="212"/>
-        <v>0.35549089809848899</v>
-      </c>
-      <c r="J338" s="272">
-        <f t="shared" si="212"/>
-        <v>0.38088547361253239</v>
-      </c>
-      <c r="K338" s="272">
-        <f t="shared" si="212"/>
-        <v>0.43333887196009591</v>
-      </c>
-    </row>
-    <row r="339" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="D339" s="272"/>
-      <c r="E339" s="272"/>
-      <c r="F339" s="272"/>
-      <c r="G339" s="272"/>
-      <c r="H339" s="272"/>
-      <c r="I339" s="272"/>
-      <c r="J339" s="272"/>
-      <c r="K339" s="272"/>
-    </row>
-    <row r="340" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C340" s="6" t="s">
+      <c r="H343" s="272">
+        <f t="shared" si="213"/>
+        <v>0.35721699923682693</v>
+      </c>
+      <c r="I343" s="272">
+        <f t="shared" si="213"/>
+        <v>0.3537115410111874</v>
+      </c>
+      <c r="J343" s="272">
+        <f t="shared" si="213"/>
+        <v>0.37700009784494043</v>
+      </c>
+      <c r="K343" s="272">
+        <f t="shared" si="213"/>
+        <v>0.4255664579710956</v>
+      </c>
+    </row>
+    <row r="344" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="D344" s="272"/>
+      <c r="E344" s="272"/>
+      <c r="F344" s="272"/>
+      <c r="G344" s="272"/>
+      <c r="H344" s="272"/>
+      <c r="I344" s="272"/>
+      <c r="J344" s="272"/>
+      <c r="K344" s="272"/>
+    </row>
+    <row r="345" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C345" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="D345" s="272"/>
+      <c r="E345" s="272"/>
+      <c r="F345" s="272"/>
+      <c r="G345" s="272"/>
+      <c r="H345" s="272"/>
+      <c r="I345" s="272"/>
+      <c r="J345" s="272"/>
+      <c r="K345" s="272"/>
+    </row>
+    <row r="346" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C346" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="D346" s="1">
+        <f>D28/D72</f>
+        <v>5.6681443050736427E-2</v>
+      </c>
+      <c r="E346" s="1">
+        <f t="shared" ref="E346:K346" si="214">E28/E72</f>
+        <v>6.5049190338720572E-2</v>
+      </c>
+      <c r="F346" s="1">
+        <f t="shared" si="214"/>
+        <v>6.1467692589002032E-2</v>
+      </c>
+      <c r="G346" s="1">
+        <f t="shared" si="214"/>
+        <v>5.970788857829646E-2</v>
+      </c>
+      <c r="H346" s="1">
+        <f t="shared" si="214"/>
+        <v>5.8532242769790702E-2</v>
+      </c>
+      <c r="I346" s="1">
+        <f t="shared" si="214"/>
+        <v>5.8725926164176823E-2</v>
+      </c>
+      <c r="J346" s="1">
+        <f t="shared" si="214"/>
+        <v>5.9470596354519394E-2</v>
+      </c>
+      <c r="K346" s="1">
+        <f t="shared" si="214"/>
+        <v>6.067908338471658E-2</v>
+      </c>
+    </row>
+    <row r="347" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C347" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="D347" s="1">
+        <f>D28/D105</f>
+        <v>0.11519732492177333</v>
+      </c>
+      <c r="E347" s="1">
+        <f t="shared" ref="E347:K347" si="215">E28/E105</f>
+        <v>0.12312547216421023</v>
+      </c>
+      <c r="F347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.11967870394241095</v>
+      </c>
+      <c r="G347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.11836700091904881</v>
+      </c>
+      <c r="H347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.1179256291247</v>
+      </c>
+      <c r="I347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.1162781028239655</v>
+      </c>
+      <c r="J347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.11390530414541496</v>
+      </c>
+      <c r="K347" s="1">
+        <f t="shared" si="215"/>
+        <v>0.11138576335644054</v>
+      </c>
+    </row>
+    <row r="349" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C349" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="D349" s="272"/>
+      <c r="E349" s="272"/>
+      <c r="F349" s="272"/>
+      <c r="G349" s="272"/>
+      <c r="H349" s="272"/>
+      <c r="I349" s="272"/>
+      <c r="J349" s="272"/>
+      <c r="K349" s="272"/>
+    </row>
+    <row r="350" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C350" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="D350" s="217">
+        <f>D28/D16</f>
+        <v>0.10480039293844859</v>
+      </c>
+      <c r="E350" s="217">
+        <f t="shared" ref="E350:K350" si="216">E28/E16</f>
+        <v>0.11028221247472296</v>
+      </c>
+      <c r="F350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11133862705595989</v>
+      </c>
+      <c r="G350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11196914563644411</v>
+      </c>
+      <c r="H350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11313214563362482</v>
+      </c>
+      <c r="I350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11406135045663253</v>
+      </c>
+      <c r="J350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11483067091070658</v>
+      </c>
+      <c r="K350" s="217">
+        <f t="shared" si="216"/>
+        <v>0.11552307536025366</v>
+      </c>
+    </row>
+    <row r="351" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C351" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="D351" s="272">
+        <f>D16/D72</f>
+        <v>0.54085143634935229</v>
+      </c>
+      <c r="E351" s="272">
+        <f t="shared" ref="E351:K351" si="217">E16/E72</f>
+        <v>0.58984299352563374</v>
+      </c>
+      <c r="F351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.5520787727884211</v>
+      </c>
+      <c r="G351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.5332530514447591</v>
+      </c>
+      <c r="H351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.51737941008690558</v>
+      </c>
+      <c r="I351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.51486262374655223</v>
+      </c>
+      <c r="J351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.517898187678136</v>
+      </c>
+      <c r="K351" s="272">
+        <f t="shared" si="217"/>
+        <v>0.52525509034010309</v>
+      </c>
+    </row>
+    <row r="352" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C352" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="D352" s="272">
+        <f>D72/D105</f>
+        <v>2.0323640105397183</v>
+      </c>
+      <c r="E352" s="272">
+        <f t="shared" ref="E352:K352" si="218">E72/E105</f>
+        <v>1.8928056063892267</v>
+      </c>
+      <c r="F352" s="272">
+        <f t="shared" si="218"/>
+        <v>1.9470180008648021</v>
+      </c>
+      <c r="G352" s="272">
+        <f t="shared" si="218"/>
+        <v>1.9824348798372124</v>
+      </c>
+      <c r="H352" s="272">
+        <f t="shared" si="218"/>
+        <v>2.0147122943589486</v>
+      </c>
+      <c r="I352" s="272">
+        <f t="shared" si="218"/>
+        <v>1.9800130950492505</v>
+      </c>
+      <c r="J352" s="272">
+        <f t="shared" si="218"/>
+        <v>1.9153213710250423</v>
+      </c>
+      <c r="K352" s="272">
+        <f t="shared" si="218"/>
+        <v>1.8356533609816459</v>
+      </c>
+    </row>
+    <row r="353" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C353" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="D353" s="1">
+        <f>D350*D351*D352</f>
+        <v>0.11519732492177334</v>
+      </c>
+      <c r="E353" s="1">
+        <f t="shared" ref="E353:K353" si="219">E350*E351*E352</f>
+        <v>0.12312547216421024</v>
+      </c>
+      <c r="F353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.11967870394241095</v>
+      </c>
+      <c r="G353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.1183670009190488</v>
+      </c>
+      <c r="H353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.1179256291247</v>
+      </c>
+      <c r="I353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.11627810282396553</v>
+      </c>
+      <c r="J353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.11390530414541496</v>
+      </c>
+      <c r="K353" s="1">
+        <f t="shared" si="219"/>
+        <v>0.11138576335644053</v>
+      </c>
+    </row>
+    <row r="354" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C354" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="D354" s="191">
+        <f>D353-D347</f>
+        <v>0</v>
+      </c>
+      <c r="E354" s="191">
+        <f t="shared" ref="E354:K354" si="220">E353-E347</f>
+        <v>0</v>
+      </c>
+      <c r="F354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+      <c r="G354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+      <c r="H354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+      <c r="I354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+      <c r="J354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+      <c r="K354" s="191">
+        <f t="shared" si="220"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C356" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="D340" s="30" t="str">
-        <f>IF(AND(D333&lt;1.5, D338&gt;1), "Strong", IF(D333&lt;3, "Adequate", "Elevated"))</f>
+      <c r="D356" s="30" t="str">
+        <f t="shared" ref="D356:K356" si="221">IF(AND(D334&lt;1.5, D343&gt;1), "Strong", IF(D334&lt;3, "Adequate", "Elevated"))</f>
         <v>Adequate</v>
       </c>
-      <c r="E340" s="30" t="str">
-        <f t="shared" ref="E340:K340" si="213">IF(AND(E333&lt;1.5, E338&gt;1), "Strong", IF(E333&lt;3, "Adequate", "Elevated"))</f>
+      <c r="E356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="F340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="F356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="G340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="G356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="H340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="H356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="I340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="I356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="J340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="J356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
-      <c r="K340" s="30" t="str">
-        <f t="shared" si="213"/>
+      <c r="K356" s="30" t="str">
+        <f t="shared" si="221"/>
         <v>Adequate</v>
       </c>
     </row>

</xml_diff>